<commit_message>
Added Funds Tranfers Test Cases
</commit_message>
<xml_diff>
--- a/TestData/Bank_of_america_all_accounts.xlsx
+++ b/TestData/Bank_of_america_all_accounts.xlsx
@@ -439,7 +439,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Saving Account</t>
+          <t>667</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -464,7 +464,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Current Account</t>
+          <t>128</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Saving Account</t>
+          <t>21</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Current Account</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Saving Account</t>
+          <t>83</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Saving Account</t>
+          <t>83</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Current Account</t>
+          <t>128</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>

<commit_message>
Added Bill CustomerSupport.py and Transaction_History.py Test Cases
</commit_message>
<xml_diff>
--- a/TestData/Bank_of_america_all_accounts.xlsx
+++ b/TestData/Bank_of_america_all_accounts.xlsx
@@ -439,12 +439,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>667</t>
+          <t>Saving Account</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>3000087</t>
+          <t>2984926</t>
         </is>
       </c>
     </row>
@@ -464,7 +464,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>Current Account</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -489,7 +489,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>Saving Account</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -514,7 +514,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Current Account</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>Saving Account</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>Saving Account</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -589,7 +589,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>Current Account</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">

</xml_diff>